<commit_message>
style: wrap scanner tables and import preview in scrollable divs; clean checkin status columns and scanned logs
</commit_message>
<xml_diff>
--- a/data_test.xlsx
+++ b/data_test.xlsx
@@ -624,11 +624,6 @@
 ID: I2MVJV1Q</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Scanned</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="75" customHeight="1">
       <c r="A3" t="inlineStr">

</xml_diff>